<commit_message>
feat(validation): update Excel workbook and Google Apps Script to English for European consortium
</commit_message>
<xml_diff>
--- a/public/documents/validation/Learning_Brains_Training_Itinerary_Validation_Responses.xlsx
+++ b/public/documents/validation/Learning_Brains_Training_Itinerary_Validation_Responses.xlsx
@@ -7,12 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Respuestas_Itinerario" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook_Preguntas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation_Responses" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook_Questions" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI_Dashboard" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Respuestas_Itinerario'!$A$2:$AU$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Validation_Responses'!$A$2:$AU$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -54,13 +54,12 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="14"/>
+      <sz val="13"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="13"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -247,9 +246,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
@@ -648,57 +645,57 @@
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
-    <col width="12" customWidth="1" min="22" max="22"/>
-    <col width="12" customWidth="1" min="23" max="23"/>
-    <col width="12" customWidth="1" min="24" max="24"/>
-    <col width="12" customWidth="1" min="25" max="25"/>
-    <col width="12" customWidth="1" min="26" max="26"/>
-    <col width="12" customWidth="1" min="27" max="27"/>
-    <col width="12" customWidth="1" min="28" max="28"/>
-    <col width="12" customWidth="1" min="29" max="29"/>
-    <col width="12" customWidth="1" min="30" max="30"/>
-    <col width="12" customWidth="1" min="31" max="31"/>
-    <col width="12" customWidth="1" min="32" max="32"/>
-    <col width="12" customWidth="1" min="33" max="33"/>
-    <col width="12" customWidth="1" min="34" max="34"/>
-    <col width="12" customWidth="1" min="35" max="35"/>
-    <col width="12" customWidth="1" min="36" max="36"/>
-    <col width="12" customWidth="1" min="37" max="37"/>
-    <col width="14" customWidth="1" min="38" max="38"/>
-    <col width="14" customWidth="1" min="39" max="39"/>
-    <col width="14" customWidth="1" min="40" max="40"/>
-    <col width="14" customWidth="1" min="41" max="41"/>
-    <col width="14" customWidth="1" min="42" max="42"/>
-    <col width="14" customWidth="1" min="43" max="43"/>
-    <col width="15" customWidth="1" min="44" max="44"/>
-    <col width="40" customWidth="1" min="45" max="45"/>
-    <col width="40" customWidth="1" min="46" max="46"/>
-    <col width="40" customWidth="1" min="47" max="47"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="13" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="13" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="25" max="25"/>
+    <col width="13" customWidth="1" min="26" max="26"/>
+    <col width="13" customWidth="1" min="27" max="27"/>
+    <col width="13" customWidth="1" min="28" max="28"/>
+    <col width="13" customWidth="1" min="29" max="29"/>
+    <col width="13" customWidth="1" min="30" max="30"/>
+    <col width="13" customWidth="1" min="31" max="31"/>
+    <col width="13" customWidth="1" min="32" max="32"/>
+    <col width="13" customWidth="1" min="33" max="33"/>
+    <col width="13" customWidth="1" min="34" max="34"/>
+    <col width="13" customWidth="1" min="35" max="35"/>
+    <col width="13" customWidth="1" min="36" max="36"/>
+    <col width="13" customWidth="1" min="37" max="37"/>
+    <col width="15" customWidth="1" min="38" max="38"/>
+    <col width="15" customWidth="1" min="39" max="39"/>
+    <col width="15" customWidth="1" min="40" max="40"/>
+    <col width="15" customWidth="1" min="41" max="41"/>
+    <col width="15" customWidth="1" min="42" max="42"/>
+    <col width="15" customWidth="1" min="43" max="43"/>
+    <col width="16" customWidth="1" min="44" max="44"/>
+    <col width="42" customWidth="1" min="45" max="45"/>
+    <col width="42" customWidth="1" min="46" max="46"/>
+    <col width="42" customWidth="1" min="47" max="47"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>1. METADATOS Y PERFIL DEL EVALUADOR / METADATA &amp; EVALUATOR PROFILE</t>
+          <t>1. METADATA &amp; EVALUATOR PROFILE</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -713,7 +710,7 @@
       <c r="K1" s="2" t="n"/>
       <c r="L1" s="3" t="inlineStr">
         <is>
-          <t>2. OBJETO Y PERTINENCIA / PURPOSE &amp; RELEVANCE (P1-P4)</t>
+          <t>2. PURPOSE &amp; RELEVANCE (P1-P4)</t>
         </is>
       </c>
       <c r="M1" s="4" t="n"/>
@@ -721,7 +718,7 @@
       <c r="O1" s="4" t="n"/>
       <c r="P1" s="5" t="inlineStr">
         <is>
-          <t>3. ESTRUCTURA Y COHERENCIA / STRUCTURE &amp; COHERENCE (S1-S4)</t>
+          <t>3. STRUCTURE &amp; COHERENCE (S1-S4)</t>
         </is>
       </c>
       <c r="Q1" s="6" t="n"/>
@@ -729,7 +726,7 @@
       <c r="S1" s="6" t="n"/>
       <c r="T1" s="7" t="inlineStr">
         <is>
-          <t>4. UNIDADES DE APRENDIZAJE / LEARNING UNITS (U1-U5)</t>
+          <t>4. LEARNING UNITS (U1-U5)</t>
         </is>
       </c>
       <c r="U1" s="8" t="n"/>
@@ -738,7 +735,7 @@
       <c r="X1" s="8" t="n"/>
       <c r="Y1" s="9" t="inlineStr">
         <is>
-          <t>5. PRINCIPIOS ÉTICOS Y LEGALES / ETHICS &amp; INCLUSION (E1-E4)</t>
+          <t>5. ETHICAL &amp; LEGAL PRINCIPLES (E1-E4)</t>
         </is>
       </c>
       <c r="Z1" s="10" t="n"/>
@@ -746,7 +743,7 @@
       <c r="AB1" s="10" t="n"/>
       <c r="AC1" s="11" t="inlineStr">
         <is>
-          <t>6. MARCO DE COMPETENCIAS / COMPETENCE FRAMEWORK (C1-C4)</t>
+          <t>6. COMPETENCE FRAMEWORK (C1-C4)</t>
         </is>
       </c>
       <c r="AD1" s="12" t="n"/>
@@ -754,7 +751,7 @@
       <c r="AF1" s="12" t="n"/>
       <c r="AG1" s="13" t="inlineStr">
         <is>
-          <t>7. USO PRÁCTICO Y TRANSFERIBILIDAD / PRACTICAL USE &amp; TRANSFER (T1-T5)</t>
+          <t>7. PRACTICAL USE &amp; TRANSFERABILITY (T1-T5)</t>
         </is>
       </c>
       <c r="AH1" s="14" t="n"/>
@@ -763,7 +760,7 @@
       <c r="AK1" s="14" t="n"/>
       <c r="AL1" s="15" t="inlineStr">
         <is>
-          <t>PROMEDIOS CALCULADOS (1-5) / CALCULATED AVERAGES</t>
+          <t>CALCULATED SECTION AVERAGES (1-5)</t>
         </is>
       </c>
       <c r="AM1" s="16" t="n"/>
@@ -774,7 +771,7 @@
       <c r="AR1" s="16" t="n"/>
       <c r="AS1" s="17" t="inlineStr">
         <is>
-          <t>8. COMENTARIOS CUALITATIVOS / QUALITATIVE FEEDBACK</t>
+          <t>8. QUALITATIVE FEEDBACK (OPEN COMMENTS)</t>
         </is>
       </c>
       <c r="AT1" s="18" t="n"/>
@@ -784,282 +781,283 @@
       <c r="A2" s="19" t="inlineStr">
         <is>
           <t>Timestamp
-(Fecha y hora (UTC))</t>
+(Submission Date (UTC))</t>
         </is>
       </c>
       <c r="B2" s="19" t="inlineStr">
         <is>
           <t>Campaign
-(ID Campaña)</t>
+(Campaign ID)</t>
         </is>
       </c>
       <c r="C2" s="19" t="inlineStr">
         <is>
           <t>Language
-(Idioma)</t>
+(Form Language)</t>
         </is>
       </c>
       <c r="D2" s="19" t="inlineStr">
         <is>
-          <t>Name
-(Nombre y Apellidos)</t>
+          <t>Full_Name
+(Evaluator Name)</t>
         </is>
       </c>
       <c r="E2" s="19" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Email
+(Evaluator Email)</t>
         </is>
       </c>
       <c r="F2" s="19" t="inlineStr">
         <is>
           <t>Organization
-(Organización / Entidad)</t>
+(Organization / Company)</t>
         </is>
       </c>
       <c r="G2" s="19" t="inlineStr">
         <is>
           <t>Country
-(País)</t>
+(Country Code)</t>
         </is>
       </c>
       <c r="H2" s="19" t="inlineStr">
         <is>
-          <t>Profile
-(Perfil Profesional)</t>
+          <t>Professional_Background
+(Professional Profile)</t>
         </is>
       </c>
       <c r="I2" s="19" t="inlineStr">
         <is>
-          <t>Other_Detail
-(Detalle otro perfil)</t>
+          <t>Other_Background_Detail
+(Other Profile Details)</t>
         </is>
       </c>
       <c r="J2" s="19" t="inlineStr">
         <is>
-          <t>Experience
-(Años Experiencia)</t>
+          <t>Experience_Years
+(Years of Experience)</t>
         </is>
       </c>
       <c r="K2" s="19" t="inlineStr">
         <is>
-          <t>AI_Level
-(Nivel Experiencia IA)</t>
+          <t>AI_Experience_Level
+(AI Experience Level)</t>
         </is>
       </c>
       <c r="L2" s="20" t="inlineStr">
         <is>
           <t>P1
-(P1: Necesidades puesto trabajo)</t>
+(P1: On-the-job training needs)</t>
         </is>
       </c>
       <c r="M2" s="20" t="inlineStr">
         <is>
           <t>P2
-(P2: Objetivos claros)</t>
+(P2: Clear overall aims)</t>
         </is>
       </c>
       <c r="N2" s="20" t="inlineStr">
         <is>
           <t>P3
-(P3: Destinatarios claros)</t>
+(P3: Clear target groups)</t>
         </is>
       </c>
       <c r="O2" s="20" t="inlineStr">
         <is>
           <t>P4
-(P4: Relevancia RRHH/formadores)</t>
+(P4: Relevance to HR &amp; trainers)</t>
         </is>
       </c>
       <c r="P2" s="21" t="inlineStr">
         <is>
           <t>S1
-(S1: Estructura clara y navegable)</t>
+(S1: Clear structure &amp; navigation)</t>
         </is>
       </c>
       <c r="Q2" s="21" t="inlineStr">
         <is>
           <t>S2
-(S2: División en 4 partes útil)</t>
+(S2: 4-part division is logical)</t>
         </is>
       </c>
       <c r="R2" s="21" t="inlineStr">
         <is>
           <t>S3
-(S3: Conexión marcos europeos)</t>
+(S3: EU frameworks alignment)</t>
         </is>
       </c>
       <c r="S2" s="21" t="inlineStr">
         <is>
           <t>S4
-(S4: Progresión coherente)</t>
+(S4: Coherent unit progression)</t>
         </is>
       </c>
       <c r="T2" s="22" t="inlineStr">
         <is>
           <t>U1
-(U1: Cobertura competencias)</t>
+(U1: AI core competences)</t>
         </is>
       </c>
       <c r="U2" s="22" t="inlineStr">
         <is>
           <t>U2
-(U2: Claridad enfoque unidades)</t>
+(U2: Clear unit core focus)</t>
         </is>
       </c>
       <c r="V2" s="22" t="inlineStr">
         <is>
           <t>U3
-(U3: Resultados realistas)</t>
+(U3: Realistic learning outcomes)</t>
         </is>
       </c>
       <c r="W2" s="22" t="inlineStr">
         <is>
           <t>U4
-(U4: Equilibrio concepto/práctica)</t>
+(U4: Concept/practice balance)</t>
         </is>
       </c>
       <c r="X2" s="22" t="inlineStr">
         <is>
           <t>U5
-(U5: Adaptable a perfiles/empresas)</t>
+(U5: Target &amp; company adaptability)</t>
         </is>
       </c>
       <c r="Y2" s="23" t="inlineStr">
         <is>
           <t>E1
-(E1: Integración ética/legal)</t>
+(E1: Ethical &amp; legal integration)</t>
         </is>
       </c>
       <c r="Z2" s="23" t="inlineStr">
         <is>
           <t>E2
-(E2: Adecuado a destinatarios)</t>
+(E2: Suitable for target groups)</t>
         </is>
       </c>
       <c r="AA2" s="23" t="inlineStr">
         <is>
           <t>E3
-(E3: Conexión selección herramientas)</t>
+(E3: Tool &amp; training connection)</t>
         </is>
       </c>
       <c r="AB2" s="23" t="inlineStr">
         <is>
           <t>E4
-(E4: Equidad e inclusión)</t>
+(E4: Fairness &amp; inclusion)</t>
         </is>
       </c>
       <c r="AC2" s="24" t="inlineStr">
         <is>
           <t>C1
-(C1: Estructura KSA adecuada)</t>
+(C1: KSA structure appropriate)</t>
         </is>
       </c>
       <c r="AD2" s="24" t="inlineStr">
         <is>
           <t>C2
-(C2: Alineación con unidades)</t>
+(C2: Alignment with learning units)</t>
         </is>
       </c>
       <c r="AE2" s="24" t="inlineStr">
         <is>
           <t>C3
-(C3: Actitudes responsables IA)</t>
+(C3: Responsible AI attitudes)</t>
         </is>
       </c>
       <c r="AF2" s="24" t="inlineStr">
         <is>
           <t>C4
-(C4: Base para nuevos contenidos)</t>
+(C4: Foundation for content creation)</t>
         </is>
       </c>
       <c r="AG2" s="25" t="inlineStr">
         <is>
           <t>T1
-(T1: Guía para Programa Formativo)</t>
+(T1: Training Programme guidance)</t>
         </is>
       </c>
       <c r="AH2" s="25" t="inlineStr">
         <is>
           <t>T2
-(T2: Guía para formadores útil)</t>
+(T2: Useful trainer guidance)</t>
         </is>
       </c>
       <c r="AI2" s="25" t="inlineStr">
         <is>
           <t>T3
-(T3: Hoja de ruta adaptación)</t>
+(T3: Adaptation roadmap helpful)</t>
         </is>
       </c>
       <c r="AJ2" s="25" t="inlineStr">
         <is>
           <t>T4
-(T4: Claridad agentes externos)</t>
+(T4: Clear for external trainers)</t>
         </is>
       </c>
       <c r="AK2" s="25" t="inlineStr">
         <is>
           <t>T5
-(T5: Potencial contextos europeos)</t>
+(T5: Potential in European contexts)</t>
         </is>
       </c>
       <c r="AL2" s="26" t="inlineStr">
         <is>
-          <t>Media_P
-(Media Sec 2 (Objeto))</t>
+          <t>Mean_Sec2
+(Mean Sec 2: Purpose)</t>
         </is>
       </c>
       <c r="AM2" s="26" t="inlineStr">
         <is>
-          <t>Media_S
-(Media Sec 3 (Estructura))</t>
+          <t>Mean_Sec3
+(Mean Sec 3: Structure)</t>
         </is>
       </c>
       <c r="AN2" s="26" t="inlineStr">
         <is>
-          <t>Media_U
-(Media Sec 4 (Unidades))</t>
+          <t>Mean_Sec4
+(Mean Sec 4: Units)</t>
         </is>
       </c>
       <c r="AO2" s="26" t="inlineStr">
         <is>
-          <t>Media_E
-(Media Sec 5 (Ética))</t>
+          <t>Mean_Sec5
+(Mean Sec 5: Ethics)</t>
         </is>
       </c>
       <c r="AP2" s="26" t="inlineStr">
         <is>
-          <t>Media_C
-(Media Sec 6 (Competencias))</t>
+          <t>Mean_Sec6
+(Mean Sec 6: Competences)</t>
         </is>
       </c>
       <c r="AQ2" s="26" t="inlineStr">
         <is>
-          <t>Media_T
-(Media Sec 7 (Transferencia))</t>
+          <t>Mean_Sec7
+(Mean Sec 7: Transfer)</t>
         </is>
       </c>
       <c r="AR2" s="26" t="inlineStr">
         <is>
-          <t>Media_Global
-(Media Global (1-5))</t>
+          <t>Overall_Mean
+(Overall Mean Score (1-5))</t>
         </is>
       </c>
       <c r="AS2" s="27" t="inlineStr">
         <is>
           <t>Q1_Strengths
-(Q1: Puntos fuertes principales)</t>
+(Q1: Main Strengths of Itinerary)</t>
         </is>
       </c>
       <c r="AT2" s="27" t="inlineStr">
         <is>
           <t>Q2_Improvements
-(Q2: Aspectos a revisar o mejorar)</t>
+(Q2: Aspects to Revise / Improve)</t>
         </is>
       </c>
       <c r="AU2" s="27" t="inlineStr">
         <is>
           <t>Q3_Missing_Topics
-(Q3: Temas o competencias ausentes)</t>
+(Q3: Missing Topics / Competences)</t>
         </is>
       </c>
     </row>
@@ -1076,22 +1074,22 @@
       </c>
       <c r="C3" s="28" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>EN</t>
         </is>
       </c>
       <c r="D3" s="29" t="inlineStr">
         <is>
-          <t>Ejemplo Evaluador</t>
+          <t>Sample Evaluator</t>
         </is>
       </c>
       <c r="E3" s="29" t="inlineStr">
         <is>
-          <t>evaluador@ejemplo.eu</t>
+          <t>evaluator@example.eu</t>
         </is>
       </c>
       <c r="F3" s="29" t="inlineStr">
         <is>
-          <t>Centro FP Industrial / Empresa</t>
+          <t>Industrial Training Center / SME</t>
         </is>
       </c>
       <c r="G3" s="28" t="inlineStr">
@@ -1223,17 +1221,17 @@
       </c>
       <c r="AS3" s="31" t="inlineStr">
         <is>
-          <t>Excelente estructuración de las 6 unidades formativas y gran aplicabilidad en PYMEs.</t>
+          <t>Excellent structure of the 6 learning units with immediate applicability to industrial SMEs.</t>
         </is>
       </c>
       <c r="AT3" s="31" t="inlineStr">
         <is>
-          <t>Reforzar con ejemplos concretos de prompts en el módulo de herramientas industriales.</t>
+          <t>Include more real-world prompting templates for industrial inspection in Unit 3.</t>
         </is>
       </c>
       <c r="AU3" s="31" t="inlineStr">
         <is>
-          <t>Ninguno en particular, el itinerario es muy completo.</t>
+          <t>None, the itinerary provides a very comprehensive foundation.</t>
         </is>
       </c>
     </row>
@@ -1260,47 +1258,47 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="32" t="inlineStr">
         <is>
-          <t>LEARNING BRAINS (ERASMUS+) - CODEBOOK Y DICCIONARIO DE VARIABLES</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="24" customHeight="1">
+          <t>LEARNING BRAINS (ERASMUS+) - VALIDATION CODEBOOK &amp; VARIABLE DICTIONARY</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="26" customHeight="1">
       <c r="A3" s="33" t="inlineStr">
         <is>
-          <t>Código</t>
+          <t>Item Code</t>
         </is>
       </c>
       <c r="B3" s="34" t="inlineStr">
         <is>
-          <t>Sección</t>
+          <t>Section Name</t>
         </is>
       </c>
       <c r="C3" s="34" t="inlineStr">
         <is>
-          <t>Pregunta en Inglés (Original)</t>
+          <t>Official Question Text (English)</t>
         </is>
       </c>
       <c r="D3" s="34" t="inlineStr">
         <is>
-          <t>Pregunta en Español</t>
+          <t>Question Text (Spanish Reference)</t>
         </is>
       </c>
       <c r="E3" s="33" t="inlineStr">
         <is>
-          <t>Escala / Tipo</t>
+          <t>Scale / Response Type</t>
         </is>
       </c>
     </row>
@@ -1312,7 +1310,7 @@
       </c>
       <c r="B4" s="29" t="inlineStr">
         <is>
-          <t>Sección 2: Objeto y pertinencia</t>
+          <t>Section 2. Purpose and relevance</t>
         </is>
       </c>
       <c r="C4" s="29" t="inlineStr">
@@ -1327,7 +1325,7 @@
       </c>
       <c r="E4" s="28" t="inlineStr">
         <is>
-          <t>Likert (1-5)</t>
+          <t>Likert Scale (1 - 5)</t>
         </is>
       </c>
     </row>
@@ -1339,7 +1337,7 @@
       </c>
       <c r="B5" s="29" t="inlineStr">
         <is>
-          <t>Sección 2: Objeto y pertinencia</t>
+          <t>Section 2. Purpose and relevance</t>
         </is>
       </c>
       <c r="C5" s="29" t="inlineStr">
@@ -1354,7 +1352,7 @@
       </c>
       <c r="E5" s="28" t="inlineStr">
         <is>
-          <t>Likert (1-5)</t>
+          <t>Likert Scale (1 - 5)</t>
         </is>
       </c>
     </row>
@@ -1366,7 +1364,7 @@
       </c>
       <c r="B6" s="29" t="inlineStr">
         <is>
-          <t>Sección 2: Objeto y pertinencia</t>
+          <t>Section 2. Purpose and relevance</t>
         </is>
       </c>
       <c r="C6" s="29" t="inlineStr">
@@ -1381,7 +1379,7 @@
       </c>
       <c r="E6" s="28" t="inlineStr">
         <is>
-          <t>Likert (1-5)</t>
+          <t>Likert Scale (1 - 5)</t>
         </is>
       </c>
     </row>
@@ -1393,7 +1391,7 @@
       </c>
       <c r="B7" s="29" t="inlineStr">
         <is>
-          <t>Sección 2: Objeto y pertinencia</t>
+          <t>Section 2. Purpose and relevance</t>
         </is>
       </c>
       <c r="C7" s="29" t="inlineStr">
@@ -1408,7 +1406,7 @@
       </c>
       <c r="E7" s="28" t="inlineStr">
         <is>
-          <t>Likert (1-5)</t>
+          <t>Likert Scale (1 - 5)</t>
         </is>
       </c>
     </row>
@@ -1420,7 +1418,7 @@
       </c>
       <c r="B8" s="29" t="inlineStr">
         <is>
-          <t>Sección 3: Estructura y coherencia</t>
+          <t>Section 3. Structure and coherence</t>
         </is>
       </c>
       <c r="C8" s="29" t="inlineStr">
@@ -1435,7 +1433,7 @@
       </c>
       <c r="E8" s="28" t="inlineStr">
         <is>
-          <t>Likert (1-5)</t>
+          <t>Likert Scale (1 - 5)</t>
         </is>
       </c>
     </row>
@@ -1447,7 +1445,7 @@
       </c>
       <c r="B9" s="29" t="inlineStr">
         <is>
-          <t>Sección 3: Estructura y coherencia</t>
+          <t>Section 3. Structure and coherence</t>
         </is>
       </c>
       <c r="C9" s="29" t="inlineStr">
@@ -1462,7 +1460,7 @@
       </c>
       <c r="E9" s="28" t="inlineStr">
         <is>
-          <t>Likert (1-5)</t>
+          <t>Likert Scale (1 - 5)</t>
         </is>
       </c>
     </row>
@@ -1474,7 +1472,7 @@
       </c>
       <c r="B10" s="29" t="inlineStr">
         <is>
-          <t>Sección 3: Estructura y coherencia</t>
+          <t>Section 3. Structure and coherence</t>
         </is>
       </c>
       <c r="C10" s="29" t="inlineStr">
@@ -1489,7 +1487,7 @@
       </c>
       <c r="E10" s="28" t="inlineStr">
         <is>
-          <t>Likert (1-5)</t>
+          <t>Likert Scale (1 - 5)</t>
         </is>
       </c>
     </row>
@@ -1501,7 +1499,7 @@
       </c>
       <c r="B11" s="29" t="inlineStr">
         <is>
-          <t>Sección 3: Estructura y coherencia</t>
+          <t>Section 3. Structure and coherence</t>
         </is>
       </c>
       <c r="C11" s="29" t="inlineStr">
@@ -1516,7 +1514,7 @@
       </c>
       <c r="E11" s="28" t="inlineStr">
         <is>
-          <t>Likert (1-5)</t>
+          <t>Likert Scale (1 - 5)</t>
         </is>
       </c>
     </row>
@@ -1528,7 +1526,7 @@
       </c>
       <c r="B12" s="29" t="inlineStr">
         <is>
-          <t>Sección 4: Unidades de aprendizaje</t>
+          <t>Section 4. Learning units</t>
         </is>
       </c>
       <c r="C12" s="29" t="inlineStr">
@@ -1543,7 +1541,7 @@
       </c>
       <c r="E12" s="28" t="inlineStr">
         <is>
-          <t>Likert (1-5)</t>
+          <t>Likert Scale (1 - 5)</t>
         </is>
       </c>
     </row>
@@ -1555,7 +1553,7 @@
       </c>
       <c r="B13" s="29" t="inlineStr">
         <is>
-          <t>Sección 4: Unidades de aprendizaje</t>
+          <t>Section 4. Learning units</t>
         </is>
       </c>
       <c r="C13" s="29" t="inlineStr">
@@ -1570,7 +1568,7 @@
       </c>
       <c r="E13" s="28" t="inlineStr">
         <is>
-          <t>Likert (1-5)</t>
+          <t>Likert Scale (1 - 5)</t>
         </is>
       </c>
     </row>
@@ -1582,7 +1580,7 @@
       </c>
       <c r="B14" s="29" t="inlineStr">
         <is>
-          <t>Sección 4: Unidades de aprendizaje</t>
+          <t>Section 4. Learning units</t>
         </is>
       </c>
       <c r="C14" s="29" t="inlineStr">
@@ -1597,7 +1595,7 @@
       </c>
       <c r="E14" s="28" t="inlineStr">
         <is>
-          <t>Likert (1-5)</t>
+          <t>Likert Scale (1 - 5)</t>
         </is>
       </c>
     </row>
@@ -1609,7 +1607,7 @@
       </c>
       <c r="B15" s="29" t="inlineStr">
         <is>
-          <t>Sección 4: Unidades de aprendizaje</t>
+          <t>Section 4. Learning units</t>
         </is>
       </c>
       <c r="C15" s="29" t="inlineStr">
@@ -1624,7 +1622,7 @@
       </c>
       <c r="E15" s="28" t="inlineStr">
         <is>
-          <t>Likert (1-5)</t>
+          <t>Likert Scale (1 - 5)</t>
         </is>
       </c>
     </row>
@@ -1636,7 +1634,7 @@
       </c>
       <c r="B16" s="29" t="inlineStr">
         <is>
-          <t>Sección 4: Unidades de aprendizaje</t>
+          <t>Section 4. Learning units</t>
         </is>
       </c>
       <c r="C16" s="29" t="inlineStr">
@@ -1651,7 +1649,7 @@
       </c>
       <c r="E16" s="28" t="inlineStr">
         <is>
-          <t>Likert (1-5)</t>
+          <t>Likert Scale (1 - 5)</t>
         </is>
       </c>
     </row>
@@ -1663,7 +1661,7 @@
       </c>
       <c r="B17" s="29" t="inlineStr">
         <is>
-          <t>Sección 5: Principios éticos y legales</t>
+          <t>Section 5. Ethical, legal and inclusive principles</t>
         </is>
       </c>
       <c r="C17" s="29" t="inlineStr">
@@ -1678,7 +1676,7 @@
       </c>
       <c r="E17" s="28" t="inlineStr">
         <is>
-          <t>Likert (1-5)</t>
+          <t>Likert Scale (1 - 5)</t>
         </is>
       </c>
     </row>
@@ -1690,7 +1688,7 @@
       </c>
       <c r="B18" s="29" t="inlineStr">
         <is>
-          <t>Sección 5: Principios éticos y legales</t>
+          <t>Section 5. Ethical, legal and inclusive principles</t>
         </is>
       </c>
       <c r="C18" s="29" t="inlineStr">
@@ -1705,7 +1703,7 @@
       </c>
       <c r="E18" s="28" t="inlineStr">
         <is>
-          <t>Likert (1-5)</t>
+          <t>Likert Scale (1 - 5)</t>
         </is>
       </c>
     </row>
@@ -1717,7 +1715,7 @@
       </c>
       <c r="B19" s="29" t="inlineStr">
         <is>
-          <t>Sección 5: Principios éticos y legales</t>
+          <t>Section 5. Ethical, legal and inclusive principles</t>
         </is>
       </c>
       <c r="C19" s="29" t="inlineStr">
@@ -1732,7 +1730,7 @@
       </c>
       <c r="E19" s="28" t="inlineStr">
         <is>
-          <t>Likert (1-5)</t>
+          <t>Likert Scale (1 - 5)</t>
         </is>
       </c>
     </row>
@@ -1744,7 +1742,7 @@
       </c>
       <c r="B20" s="29" t="inlineStr">
         <is>
-          <t>Sección 5: Principios éticos y legales</t>
+          <t>Section 5. Ethical, legal and inclusive principles</t>
         </is>
       </c>
       <c r="C20" s="29" t="inlineStr">
@@ -1759,7 +1757,7 @@
       </c>
       <c r="E20" s="28" t="inlineStr">
         <is>
-          <t>Likert (1-5)</t>
+          <t>Likert Scale (1 - 5)</t>
         </is>
       </c>
     </row>
@@ -1771,7 +1769,7 @@
       </c>
       <c r="B21" s="29" t="inlineStr">
         <is>
-          <t>Sección 6: Marco de competencias</t>
+          <t>Section 6. Competence framework</t>
         </is>
       </c>
       <c r="C21" s="29" t="inlineStr">
@@ -1786,7 +1784,7 @@
       </c>
       <c r="E21" s="28" t="inlineStr">
         <is>
-          <t>Likert (1-5)</t>
+          <t>Likert Scale (1 - 5)</t>
         </is>
       </c>
     </row>
@@ -1798,7 +1796,7 @@
       </c>
       <c r="B22" s="29" t="inlineStr">
         <is>
-          <t>Sección 6: Marco de competencias</t>
+          <t>Section 6. Competence framework</t>
         </is>
       </c>
       <c r="C22" s="29" t="inlineStr">
@@ -1813,7 +1811,7 @@
       </c>
       <c r="E22" s="28" t="inlineStr">
         <is>
-          <t>Likert (1-5)</t>
+          <t>Likert Scale (1 - 5)</t>
         </is>
       </c>
     </row>
@@ -1825,7 +1823,7 @@
       </c>
       <c r="B23" s="29" t="inlineStr">
         <is>
-          <t>Sección 6: Marco de competencias</t>
+          <t>Section 6. Competence framework</t>
         </is>
       </c>
       <c r="C23" s="29" t="inlineStr">
@@ -1840,7 +1838,7 @@
       </c>
       <c r="E23" s="28" t="inlineStr">
         <is>
-          <t>Likert (1-5)</t>
+          <t>Likert Scale (1 - 5)</t>
         </is>
       </c>
     </row>
@@ -1852,7 +1850,7 @@
       </c>
       <c r="B24" s="29" t="inlineStr">
         <is>
-          <t>Sección 6: Marco de competencias</t>
+          <t>Section 6. Competence framework</t>
         </is>
       </c>
       <c r="C24" s="29" t="inlineStr">
@@ -1867,7 +1865,7 @@
       </c>
       <c r="E24" s="28" t="inlineStr">
         <is>
-          <t>Likert (1-5)</t>
+          <t>Likert Scale (1 - 5)</t>
         </is>
       </c>
     </row>
@@ -1879,7 +1877,7 @@
       </c>
       <c r="B25" s="29" t="inlineStr">
         <is>
-          <t>Sección 7: Uso práctico y transferencia</t>
+          <t>Section 7. Practical use and transferability</t>
         </is>
       </c>
       <c r="C25" s="29" t="inlineStr">
@@ -1894,7 +1892,7 @@
       </c>
       <c r="E25" s="28" t="inlineStr">
         <is>
-          <t>Likert (1-5)</t>
+          <t>Likert Scale (1 - 5)</t>
         </is>
       </c>
     </row>
@@ -1906,7 +1904,7 @@
       </c>
       <c r="B26" s="29" t="inlineStr">
         <is>
-          <t>Sección 7: Uso práctico y transferencia</t>
+          <t>Section 7. Practical use and transferability</t>
         </is>
       </c>
       <c r="C26" s="29" t="inlineStr">
@@ -1921,7 +1919,7 @@
       </c>
       <c r="E26" s="28" t="inlineStr">
         <is>
-          <t>Likert (1-5)</t>
+          <t>Likert Scale (1 - 5)</t>
         </is>
       </c>
     </row>
@@ -1933,7 +1931,7 @@
       </c>
       <c r="B27" s="29" t="inlineStr">
         <is>
-          <t>Sección 7: Uso práctico y transferencia</t>
+          <t>Section 7. Practical use and transferability</t>
         </is>
       </c>
       <c r="C27" s="29" t="inlineStr">
@@ -1948,7 +1946,7 @@
       </c>
       <c r="E27" s="28" t="inlineStr">
         <is>
-          <t>Likert (1-5)</t>
+          <t>Likert Scale (1 - 5)</t>
         </is>
       </c>
     </row>
@@ -1960,7 +1958,7 @@
       </c>
       <c r="B28" s="29" t="inlineStr">
         <is>
-          <t>Sección 7: Uso práctico y transferencia</t>
+          <t>Section 7. Practical use and transferability</t>
         </is>
       </c>
       <c r="C28" s="29" t="inlineStr">
@@ -1975,7 +1973,7 @@
       </c>
       <c r="E28" s="28" t="inlineStr">
         <is>
-          <t>Likert (1-5)</t>
+          <t>Likert Scale (1 - 5)</t>
         </is>
       </c>
     </row>
@@ -1987,7 +1985,7 @@
       </c>
       <c r="B29" s="29" t="inlineStr">
         <is>
-          <t>Sección 7: Uso práctico y transferencia</t>
+          <t>Section 7. Practical use and transferability</t>
         </is>
       </c>
       <c r="C29" s="29" t="inlineStr">
@@ -2002,7 +2000,7 @@
       </c>
       <c r="E29" s="28" t="inlineStr">
         <is>
-          <t>Likert (1-5)</t>
+          <t>Likert Scale (1 - 5)</t>
         </is>
       </c>
     </row>
@@ -2014,7 +2012,7 @@
       </c>
       <c r="B30" s="29" t="inlineStr">
         <is>
-          <t>Sección 8: Cualitativa</t>
+          <t>Section 8. Qualitative Feedback</t>
         </is>
       </c>
       <c r="C30" s="29" t="inlineStr">
@@ -2029,7 +2027,7 @@
       </c>
       <c r="E30" s="28" t="inlineStr">
         <is>
-          <t>Texto Abierto</t>
+          <t>Open Text</t>
         </is>
       </c>
     </row>
@@ -2041,7 +2039,7 @@
       </c>
       <c r="B31" s="29" t="inlineStr">
         <is>
-          <t>Sección 8: Cualitativa</t>
+          <t>Section 8. Qualitative Feedback</t>
         </is>
       </c>
       <c r="C31" s="29" t="inlineStr">
@@ -2056,7 +2054,7 @@
       </c>
       <c r="E31" s="28" t="inlineStr">
         <is>
-          <t>Texto Abierto</t>
+          <t>Open Text</t>
         </is>
       </c>
     </row>
@@ -2068,7 +2066,7 @@
       </c>
       <c r="B32" s="29" t="inlineStr">
         <is>
-          <t>Sección 8: Cualitativa</t>
+          <t>Section 8. Qualitative Feedback</t>
         </is>
       </c>
       <c r="C32" s="29" t="inlineStr">
@@ -2083,7 +2081,74 @@
       </c>
       <c r="E32" s="28" t="inlineStr">
         <is>
-          <t>Texto Abierto</t>
+          <t>Open Text</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="35" t="inlineStr">
+        <is>
+          <t>Likert Scale Definition (1 - 5):</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B36" s="29" t="inlineStr">
+        <is>
+          <t>Strongly Disagree / Totalmente en desacuerdo</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="28" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B37" s="29" t="inlineStr">
+        <is>
+          <t>Disagree / En desacuerdo</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="28" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B38" s="29" t="inlineStr">
+        <is>
+          <t>Neutral (Neither agree nor disagree) / Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="28" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B39" s="29" t="inlineStr">
+        <is>
+          <t>Agree / De acuerdo</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="28" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B40" s="29" t="inlineStr">
+        <is>
+          <t>Strongly Agree / Totalmente de acuerdo</t>
         </is>
       </c>
     </row>
@@ -2104,206 +2169,206 @@
   <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="35" t="inlineStr">
-        <is>
-          <t>LEARNING BRAINS - RESUMEN EJECUTIVO DE VALIDACIÓN (INDICADORES)</t>
+      <c r="A1" s="32" t="inlineStr">
+        <is>
+          <t>LEARNING BRAINS (ERASMUS+) - EXECUTIVE VALIDATION DASHBOARD</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="36" t="inlineStr">
         <is>
-          <t>Dimensión Evaluada</t>
+          <t>Evaluation Dimension / Area</t>
         </is>
       </c>
       <c r="B3" s="37" t="inlineStr">
         <is>
-          <t>Métrica</t>
+          <t>Key Metric</t>
         </is>
       </c>
       <c r="C3" s="37" t="inlineStr">
         <is>
-          <t>Rango</t>
+          <t>Score Range</t>
         </is>
       </c>
       <c r="D3" s="37" t="inlineStr">
         <is>
-          <t>Fórmula</t>
+          <t>Calculation Basis</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="29" t="inlineStr">
         <is>
-          <t>Total de Evaluaciones Recibidas</t>
+          <t>Total Completed Validations Received</t>
         </is>
       </c>
       <c r="B4" s="38">
-        <f>COUNTA(Respuestas_Itinerario!A3:A500)</f>
+        <f>COUNTA(Validation_Responses!A3:A500)</f>
         <v/>
       </c>
       <c r="C4" s="39" t="inlineStr">
         <is>
-          <t>Nº respuestas</t>
+          <t>Total Count</t>
         </is>
       </c>
       <c r="D4" s="40" t="inlineStr">
         <is>
-          <t>Recuento</t>
+          <t>Respondent entries count</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="29" t="inlineStr">
         <is>
-          <t>Media Sección 2: Objeto y Pertinencia</t>
+          <t>Section 2: Purpose &amp; Relevance Mean</t>
         </is>
       </c>
       <c r="B5" s="41">
-        <f>AVERAGE(Respuestas_Itinerario!AL3:AL500)</f>
+        <f>AVERAGE(Validation_Responses!AL3:AL500)</f>
         <v/>
       </c>
       <c r="C5" s="39" t="inlineStr">
         <is>
-          <t>1 - 5</t>
+          <t>1.00 - 5.00</t>
         </is>
       </c>
       <c r="D5" s="40" t="inlineStr">
         <is>
-          <t>Promedio P1-P4</t>
+          <t>Average of items P1 to P4</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="29" t="inlineStr">
         <is>
-          <t>Media Sección 3: Estructura y Coherencia</t>
+          <t>Section 3: Structure &amp; Coherence Mean</t>
         </is>
       </c>
       <c r="B6" s="41">
-        <f>AVERAGE(Respuestas_Itinerario!AM3:AM500)</f>
+        <f>AVERAGE(Validation_Responses!AM3:AM500)</f>
         <v/>
       </c>
       <c r="C6" s="39" t="inlineStr">
         <is>
-          <t>1 - 5</t>
+          <t>1.00 - 5.00</t>
         </is>
       </c>
       <c r="D6" s="40" t="inlineStr">
         <is>
-          <t>Promedio S1-S4</t>
+          <t>Average of items S1 to S4</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="29" t="inlineStr">
         <is>
-          <t>Media Sección 4: Unidades de Aprendizaje</t>
+          <t>Section 4: Learning Units Mean</t>
         </is>
       </c>
       <c r="B7" s="41">
-        <f>AVERAGE(Respuestas_Itinerario!AN3:AN500)</f>
+        <f>AVERAGE(Validation_Responses!AN3:AN500)</f>
         <v/>
       </c>
       <c r="C7" s="39" t="inlineStr">
         <is>
-          <t>1 - 5</t>
+          <t>1.00 - 5.00</t>
         </is>
       </c>
       <c r="D7" s="40" t="inlineStr">
         <is>
-          <t>Promedio U1-U5</t>
+          <t>Average of items U1 to U5</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="29" t="inlineStr">
         <is>
-          <t>Media Sección 5: Principios Éticos y Legales</t>
+          <t>Section 5: Ethical &amp; Legal Principles Mean</t>
         </is>
       </c>
       <c r="B8" s="41">
-        <f>AVERAGE(Respuestas_Itinerario!AO3:AO500)</f>
+        <f>AVERAGE(Validation_Responses!AO3:AO500)</f>
         <v/>
       </c>
       <c r="C8" s="39" t="inlineStr">
         <is>
-          <t>1 - 5</t>
+          <t>1.00 - 5.00</t>
         </is>
       </c>
       <c r="D8" s="40" t="inlineStr">
         <is>
-          <t>Promedio E1-E4</t>
+          <t>Average of items E1 to E4</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="29" t="inlineStr">
         <is>
-          <t>Media Sección 6: Marco de Competencias</t>
+          <t>Section 6: Competence Framework Mean</t>
         </is>
       </c>
       <c r="B9" s="41">
-        <f>AVERAGE(Respuestas_Itinerario!AP3:AP500)</f>
+        <f>AVERAGE(Validation_Responses!AP3:AP500)</f>
         <v/>
       </c>
       <c r="C9" s="39" t="inlineStr">
         <is>
-          <t>1 - 5</t>
+          <t>1.00 - 5.00</t>
         </is>
       </c>
       <c r="D9" s="40" t="inlineStr">
         <is>
-          <t>Promedio C1-C4</t>
+          <t>Average of items C1 to C4</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="29" t="inlineStr">
         <is>
-          <t>Media Sección 7: Uso Práctico y Transferencia</t>
+          <t>Section 7: Practical Use &amp; Transferability Mean</t>
         </is>
       </c>
       <c r="B10" s="41">
-        <f>AVERAGE(Respuestas_Itinerario!AQ3:AQ500)</f>
+        <f>AVERAGE(Validation_Responses!AQ3:AQ500)</f>
         <v/>
       </c>
       <c r="C10" s="39" t="inlineStr">
         <is>
-          <t>1 - 5</t>
+          <t>1.00 - 5.00</t>
         </is>
       </c>
       <c r="D10" s="40" t="inlineStr">
         <is>
-          <t>Promedio T1-T5</t>
+          <t>Average of items T1 to T5</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="42" t="inlineStr">
         <is>
-          <t>MEDIA GLOBAL DEL ITINERARIO FORMATIVO</t>
+          <t>OVERALL ITINERARY MEAN SCORE</t>
         </is>
       </c>
       <c r="B11" s="43">
-        <f>AVERAGE(Respuestas_Itinerario!AR3:AR500)</f>
+        <f>AVERAGE(Validation_Responses!AR3:AR500)</f>
         <v/>
       </c>
       <c r="C11" s="44" t="inlineStr">
         <is>
-          <t>1 - 5</t>
+          <t>1.00 - 5.00</t>
         </is>
       </c>
       <c r="D11" s="45" t="inlineStr">
         <is>
-          <t>Promedio Global (26 ítems)</t>
+          <t>Overall Mean across all 26 Likert items</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(validation): adapt web questionnaire and results collection to updated Google document
</commit_message>
<xml_diff>
--- a/public/documents/validation/Learning_Brains_Training_Itinerary_Validation_Responses.xlsx
+++ b/public/documents/validation/Learning_Brains_Training_Itinerary_Validation_Responses.xlsx
@@ -101,12 +101,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="007C3AED"/>
-        <bgColor rgb="007C3AED"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="000D9488"/>
         <bgColor rgb="000D9488"/>
       </patternFill>
@@ -115,6 +109,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00059669"/>
         <bgColor rgb="00059669"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007C3AED"/>
+        <bgColor rgb="007C3AED"/>
       </patternFill>
     </fill>
     <fill>
@@ -710,32 +710,32 @@
       <c r="K1" s="2" t="n"/>
       <c r="L1" s="3" t="inlineStr">
         <is>
-          <t>2. PURPOSE &amp; RELEVANCE (P1-P4)</t>
+          <t>2. PURPOSE &amp; RELEVANCE (P1-P5)</t>
         </is>
       </c>
       <c r="M1" s="4" t="n"/>
       <c r="N1" s="4" t="n"/>
       <c r="O1" s="4" t="n"/>
-      <c r="P1" s="5" t="inlineStr">
+      <c r="P1" s="4" t="n"/>
+      <c r="Q1" s="5" t="inlineStr">
         <is>
           <t>3. STRUCTURE &amp; COHERENCE (S1-S4)</t>
         </is>
       </c>
-      <c r="Q1" s="6" t="n"/>
       <c r="R1" s="6" t="n"/>
       <c r="S1" s="6" t="n"/>
-      <c r="T1" s="7" t="inlineStr">
-        <is>
-          <t>4. LEARNING UNITS (U1-U5)</t>
-        </is>
-      </c>
-      <c r="U1" s="8" t="n"/>
+      <c r="T1" s="6" t="n"/>
+      <c r="U1" s="7" t="inlineStr">
+        <is>
+          <t>4. LEARNING UNITS (U1-U4)</t>
+        </is>
+      </c>
       <c r="V1" s="8" t="n"/>
       <c r="W1" s="8" t="n"/>
       <c r="X1" s="8" t="n"/>
       <c r="Y1" s="9" t="inlineStr">
         <is>
-          <t>5. ETHICAL &amp; LEGAL PRINCIPLES (E1-E4)</t>
+          <t>5. COMPETENCE FRAMEWORK (C1-C4)</t>
         </is>
       </c>
       <c r="Z1" s="10" t="n"/>
@@ -743,18 +743,18 @@
       <c r="AB1" s="10" t="n"/>
       <c r="AC1" s="11" t="inlineStr">
         <is>
-          <t>6. COMPETENCE FRAMEWORK (C1-C4)</t>
+          <t>6. PRACTICAL USE &amp; TRANSFERABILITY (T1-T5)</t>
         </is>
       </c>
       <c r="AD1" s="12" t="n"/>
       <c r="AE1" s="12" t="n"/>
       <c r="AF1" s="12" t="n"/>
-      <c r="AG1" s="13" t="inlineStr">
-        <is>
-          <t>7. PRACTICAL USE &amp; TRANSFERABILITY (T1-T5)</t>
-        </is>
-      </c>
-      <c r="AH1" s="14" t="n"/>
+      <c r="AG1" s="12" t="n"/>
+      <c r="AH1" s="13" t="inlineStr">
+        <is>
+          <t>7. ETHICAL &amp; LEGAL PRINCIPLES (E1-E4)</t>
+        </is>
+      </c>
       <c r="AI1" s="14" t="n"/>
       <c r="AJ1" s="14" t="n"/>
       <c r="AK1" s="14" t="n"/>
@@ -847,193 +847,193 @@
       <c r="L2" s="20" t="inlineStr">
         <is>
           <t>P1
-(P1: On-the-job training needs)</t>
+(P1: Clear overall aims)</t>
         </is>
       </c>
       <c r="M2" s="20" t="inlineStr">
         <is>
           <t>P2
-(P2: Clear overall aims)</t>
+(P2: Realistic learning outcomes)</t>
         </is>
       </c>
       <c r="N2" s="20" t="inlineStr">
         <is>
           <t>P3
-(P3: Clear target groups)</t>
+(P3: On-the-job training needs)</t>
         </is>
       </c>
       <c r="O2" s="20" t="inlineStr">
         <is>
           <t>P4
-(P4: Relevance to HR &amp; trainers)</t>
-        </is>
-      </c>
-      <c r="P2" s="21" t="inlineStr">
+(P4: Clear target groups)</t>
+        </is>
+      </c>
+      <c r="P2" s="20" t="inlineStr">
+        <is>
+          <t>P5
+(P5: Relevance to HR &amp; trainers)</t>
+        </is>
+      </c>
+      <c r="Q2" s="21" t="inlineStr">
         <is>
           <t>S1
 (S1: Clear structure &amp; navigation)</t>
         </is>
       </c>
-      <c r="Q2" s="21" t="inlineStr">
+      <c r="R2" s="21" t="inlineStr">
         <is>
           <t>S2
 (S2: 4-part division is logical)</t>
         </is>
       </c>
-      <c r="R2" s="21" t="inlineStr">
+      <c r="S2" s="21" t="inlineStr">
         <is>
           <t>S3
-(S3: EU frameworks alignment)</t>
-        </is>
-      </c>
-      <c r="S2" s="21" t="inlineStr">
+(S3: Coherent unit progression)</t>
+        </is>
+      </c>
+      <c r="T2" s="21" t="inlineStr">
         <is>
           <t>S4
-(S4: Coherent unit progression)</t>
-        </is>
-      </c>
-      <c r="T2" s="22" t="inlineStr">
+(S4: EU frameworks alignment)</t>
+        </is>
+      </c>
+      <c r="U2" s="22" t="inlineStr">
         <is>
           <t>U1
 (U1: AI core competences)</t>
         </is>
       </c>
-      <c r="U2" s="22" t="inlineStr">
+      <c r="V2" s="22" t="inlineStr">
         <is>
           <t>U2
 (U2: Clear unit core focus)</t>
         </is>
       </c>
-      <c r="V2" s="22" t="inlineStr">
+      <c r="W2" s="22" t="inlineStr">
         <is>
           <t>U3
-(U3: Realistic learning outcomes)</t>
-        </is>
-      </c>
-      <c r="W2" s="22" t="inlineStr">
+(U3: Concept/practice balance)</t>
+        </is>
+      </c>
+      <c r="X2" s="22" t="inlineStr">
         <is>
           <t>U4
-(U4: Concept/practice balance)</t>
-        </is>
-      </c>
-      <c r="X2" s="22" t="inlineStr">
-        <is>
-          <t>U5
-(U5: Target &amp; company adaptability)</t>
+(U4: Target &amp; company adaptability)</t>
         </is>
       </c>
       <c r="Y2" s="23" t="inlineStr">
+        <is>
+          <t>C1
+(C1: KSA structure appropriate)</t>
+        </is>
+      </c>
+      <c r="Z2" s="23" t="inlineStr">
+        <is>
+          <t>C2
+(C2: Alignment with learning units)</t>
+        </is>
+      </c>
+      <c r="AA2" s="23" t="inlineStr">
+        <is>
+          <t>C3
+(C3: Responsible AI attitudes)</t>
+        </is>
+      </c>
+      <c r="AB2" s="23" t="inlineStr">
+        <is>
+          <t>C4
+(C4: Foundation for content creation)</t>
+        </is>
+      </c>
+      <c r="AC2" s="24" t="inlineStr">
+        <is>
+          <t>T1
+(T1: Training Programme guidance)</t>
+        </is>
+      </c>
+      <c r="AD2" s="24" t="inlineStr">
+        <is>
+          <t>T2
+(T2: Useful trainer guidance)</t>
+        </is>
+      </c>
+      <c r="AE2" s="24" t="inlineStr">
+        <is>
+          <t>T3
+(T3: Adaptation roadmap helpful)</t>
+        </is>
+      </c>
+      <c r="AF2" s="24" t="inlineStr">
+        <is>
+          <t>T4
+(T4: Clear for external trainers)</t>
+        </is>
+      </c>
+      <c r="AG2" s="24" t="inlineStr">
+        <is>
+          <t>T5
+(T5: Potential in European contexts)</t>
+        </is>
+      </c>
+      <c r="AH2" s="25" t="inlineStr">
         <is>
           <t>E1
 (E1: Ethical &amp; legal integration)</t>
         </is>
       </c>
-      <c r="Z2" s="23" t="inlineStr">
+      <c r="AI2" s="25" t="inlineStr">
         <is>
           <t>E2
 (E2: Suitable for target groups)</t>
         </is>
       </c>
-      <c r="AA2" s="23" t="inlineStr">
+      <c r="AJ2" s="25" t="inlineStr">
         <is>
           <t>E3
 (E3: Tool &amp; training connection)</t>
         </is>
       </c>
-      <c r="AB2" s="23" t="inlineStr">
+      <c r="AK2" s="25" t="inlineStr">
         <is>
           <t>E4
 (E4: Fairness &amp; inclusion)</t>
         </is>
       </c>
-      <c r="AC2" s="24" t="inlineStr">
-        <is>
-          <t>C1
-(C1: KSA structure appropriate)</t>
-        </is>
-      </c>
-      <c r="AD2" s="24" t="inlineStr">
-        <is>
-          <t>C2
-(C2: Alignment with learning units)</t>
-        </is>
-      </c>
-      <c r="AE2" s="24" t="inlineStr">
-        <is>
-          <t>C3
-(C3: Responsible AI attitudes)</t>
-        </is>
-      </c>
-      <c r="AF2" s="24" t="inlineStr">
-        <is>
-          <t>C4
-(C4: Foundation for content creation)</t>
-        </is>
-      </c>
-      <c r="AG2" s="25" t="inlineStr">
-        <is>
-          <t>T1
-(T1: Training Programme guidance)</t>
-        </is>
-      </c>
-      <c r="AH2" s="25" t="inlineStr">
-        <is>
-          <t>T2
-(T2: Useful trainer guidance)</t>
-        </is>
-      </c>
-      <c r="AI2" s="25" t="inlineStr">
-        <is>
-          <t>T3
-(T3: Adaptation roadmap helpful)</t>
-        </is>
-      </c>
-      <c r="AJ2" s="25" t="inlineStr">
-        <is>
-          <t>T4
-(T4: Clear for external trainers)</t>
-        </is>
-      </c>
-      <c r="AK2" s="25" t="inlineStr">
-        <is>
-          <t>T5
-(T5: Potential in European contexts)</t>
-        </is>
-      </c>
       <c r="AL2" s="26" t="inlineStr">
         <is>
           <t>Mean_Sec2
-(Mean Sec 2: Purpose)</t>
+(Mean Sec 2: Purpose (P1-P5))</t>
         </is>
       </c>
       <c r="AM2" s="26" t="inlineStr">
         <is>
           <t>Mean_Sec3
-(Mean Sec 3: Structure)</t>
+(Mean Sec 3: Structure (S1-S4))</t>
         </is>
       </c>
       <c r="AN2" s="26" t="inlineStr">
         <is>
           <t>Mean_Sec4
-(Mean Sec 4: Units)</t>
+(Mean Sec 4: Units (U1-U4))</t>
         </is>
       </c>
       <c r="AO2" s="26" t="inlineStr">
         <is>
           <t>Mean_Sec5
-(Mean Sec 5: Ethics)</t>
+(Mean Sec 5: Competences (C1-C4))</t>
         </is>
       </c>
       <c r="AP2" s="26" t="inlineStr">
         <is>
           <t>Mean_Sec6
-(Mean Sec 6: Competences)</t>
+(Mean Sec 6: Transfer (T1-T5))</t>
         </is>
       </c>
       <c r="AQ2" s="26" t="inlineStr">
         <is>
           <t>Mean_Sec7
-(Mean Sec 7: Transfer)</t>
+(Mean Sec 7: Ethics (E1-E4))</t>
         </is>
       </c>
       <c r="AR2" s="26" t="inlineStr">
@@ -1064,7 +1064,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>2026-09-22 14:30:00</t>
+          <t>2026-09-23 12:00:00</t>
         </is>
       </c>
       <c r="B3" s="28" t="inlineStr">
@@ -1192,15 +1192,15 @@
         <v>5</v>
       </c>
       <c r="AL3" s="30">
-        <f>AVERAGE(L3:O3)</f>
+        <f>AVERAGE(L3:P3)</f>
         <v/>
       </c>
       <c r="AM3" s="30">
-        <f>AVERAGE(P3:S3)</f>
+        <f>AVERAGE(Q3:T3)</f>
         <v/>
       </c>
       <c r="AN3" s="30">
-        <f>AVERAGE(T3:X3)</f>
+        <f>AVERAGE(U3:X3)</f>
         <v/>
       </c>
       <c r="AO3" s="30">
@@ -1208,11 +1208,11 @@
         <v/>
       </c>
       <c r="AP3" s="30">
-        <f>AVERAGE(AC3:AF3)</f>
+        <f>AVERAGE(AC3:AG3)</f>
         <v/>
       </c>
       <c r="AQ3" s="30">
-        <f>AVERAGE(AG3:AK3)</f>
+        <f>AVERAGE(AH3:AK3)</f>
         <v/>
       </c>
       <c r="AR3" s="30">
@@ -1238,12 +1238,12 @@
   </sheetData>
   <autoFilter ref="A2:AU3"/>
   <mergeCells count="9">
-    <mergeCell ref="P1:S1"/>
+    <mergeCell ref="AH1:AK1"/>
+    <mergeCell ref="U1:X1"/>
+    <mergeCell ref="L1:P1"/>
+    <mergeCell ref="AC1:AG1"/>
     <mergeCell ref="AS1:AU1"/>
-    <mergeCell ref="AC1:AF1"/>
-    <mergeCell ref="AG1:AK1"/>
-    <mergeCell ref="T1:X1"/>
-    <mergeCell ref="L1:O1"/>
+    <mergeCell ref="Q1:T1"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="Y1:AB1"/>
     <mergeCell ref="AL1:AR1"/>
@@ -1258,11 +1258,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
@@ -1315,12 +1315,12 @@
       </c>
       <c r="C4" s="29" t="inlineStr">
         <is>
-          <t>The itinerary addresses relevant needs related to on-the-job training in industrial companies.</t>
+          <t>The overall aims of the itinerary are clear.</t>
         </is>
       </c>
       <c r="D4" s="29" t="inlineStr">
         <is>
-          <t>El itinerario responde a necesidades relevantes relacionadas con el aprendizaje en el puesto de trabajo en empresas industriales.</t>
+          <t>Los objetivos generales del itinerario son claros.</t>
         </is>
       </c>
       <c r="E4" s="28" t="inlineStr">
@@ -1342,12 +1342,12 @@
       </c>
       <c r="C5" s="29" t="inlineStr">
         <is>
-          <t>The overall aims of the itinerary are clear.</t>
+          <t>The main learning outcomes are realistic and appropriate.</t>
         </is>
       </c>
       <c r="D5" s="29" t="inlineStr">
         <is>
-          <t>Los objetivos generales del itinerario son claros.</t>
+          <t>Los principales resultados de aprendizaje previstos son realistas y adecuados.</t>
         </is>
       </c>
       <c r="E5" s="28" t="inlineStr">
@@ -1369,12 +1369,12 @@
       </c>
       <c r="C6" s="29" t="inlineStr">
         <is>
-          <t>The intended target groups are clearly identified.</t>
+          <t>The itinerary addresses relevant needs related to on-the-job training in industrial companies.</t>
         </is>
       </c>
       <c r="D6" s="29" t="inlineStr">
         <is>
-          <t>Los grupos destinatarios previstos están claramente identificados.</t>
+          <t>El itinerario responde a necesidades relevantes relacionadas con el aprendizaje en el puesto de trabajo en empresas industriales.</t>
         </is>
       </c>
       <c r="E6" s="28" t="inlineStr">
@@ -1396,12 +1396,12 @@
       </c>
       <c r="C7" s="29" t="inlineStr">
         <is>
-          <t>The itinerary is relevant to HR and training managers and identified target groups.</t>
+          <t>The intended target groups are clearly identified.</t>
         </is>
       </c>
       <c r="D7" s="29" t="inlineStr">
         <is>
-          <t>El itinerario es relevante para los responsables de RRHH, formadores y los grupos destinatarios identificados.</t>
+          <t>Los grupos destinatarios previstos están claramente identificados.</t>
         </is>
       </c>
       <c r="E7" s="28" t="inlineStr">
@@ -1413,22 +1413,22 @@
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>P5</t>
         </is>
       </c>
       <c r="B8" s="29" t="inlineStr">
         <is>
-          <t>Section 3. Structure and coherence</t>
+          <t>Section 2. Purpose and relevance</t>
         </is>
       </c>
       <c r="C8" s="29" t="inlineStr">
         <is>
-          <t>The document is clearly structured and easy to navigate.</t>
+          <t>The itinerary is relevant to HR and training managers and identified target groups.</t>
         </is>
       </c>
       <c r="D8" s="29" t="inlineStr">
         <is>
-          <t>El documento está claramente estructurado y es fácil de navegar y consultar.</t>
+          <t>El itinerario es relevante para los responsables de RRHH, formadores y los grupos destinatarios identificados.</t>
         </is>
       </c>
       <c r="E8" s="28" t="inlineStr">
@@ -1440,7 +1440,7 @@
     <row r="9">
       <c r="A9" s="28" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="B9" s="29" t="inlineStr">
@@ -1450,12 +1450,12 @@
       </c>
       <c r="C9" s="29" t="inlineStr">
         <is>
-          <t>The division of the document into four parts is useful and logical.</t>
+          <t>The document is clearly structured and easy to navigate.</t>
         </is>
       </c>
       <c r="D9" s="29" t="inlineStr">
         <is>
-          <t>La división del documento en cuatro partes es útil y lógica.</t>
+          <t>El documento está claramente estructurado y es fácil de navegar y consultar.</t>
         </is>
       </c>
       <c r="E9" s="28" t="inlineStr">
@@ -1467,7 +1467,7 @@
     <row r="10">
       <c r="A10" s="28" t="inlineStr">
         <is>
-          <t>S3</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="B10" s="29" t="inlineStr">
@@ -1477,12 +1477,12 @@
       </c>
       <c r="C10" s="29" t="inlineStr">
         <is>
-          <t>The relationship between the framework, the learning units, the guidance for trainers and the European reference frameworks is clear.</t>
+          <t>The division of the document into four parts is useful and logical.</t>
         </is>
       </c>
       <c r="D10" s="29" t="inlineStr">
         <is>
-          <t>La relación entre el marco, las unidades de aprendizaje, la guía para formadores y los marcos de referencia europeos es clara.</t>
+          <t>La división del documento en cuatro partes es útil y lógica.</t>
         </is>
       </c>
       <c r="E10" s="28" t="inlineStr">
@@ -1494,7 +1494,7 @@
     <row r="11">
       <c r="A11" s="28" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>S3</t>
         </is>
       </c>
       <c r="B11" s="29" t="inlineStr">
@@ -1521,22 +1521,22 @@
     <row r="12">
       <c r="A12" s="28" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>S4</t>
         </is>
       </c>
       <c r="B12" s="29" t="inlineStr">
         <is>
-          <t>Section 4. Learning units</t>
+          <t>Section 3. Structure and coherence</t>
         </is>
       </c>
       <c r="C12" s="29" t="inlineStr">
         <is>
-          <t>The six learning units collectively cover the main competences needed to use AI in on-the-job training.</t>
+          <t>The relationship between the framework, the learning units, the guidance for trainers and the European reference frameworks is clear.</t>
         </is>
       </c>
       <c r="D12" s="29" t="inlineStr">
         <is>
-          <t>Las seis unidades de aprendizaje cubren en conjunto las principales competencias necesarias para utilizar la IA en la formación en el puesto de trabajo.</t>
+          <t>La relación entre el marco, las unidades de aprendizaje, la guía para formadores y los marcos de referencia europeos es clara.</t>
         </is>
       </c>
       <c r="E12" s="28" t="inlineStr">
@@ -1548,7 +1548,7 @@
     <row r="13">
       <c r="A13" s="28" t="inlineStr">
         <is>
-          <t>U2</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="B13" s="29" t="inlineStr">
@@ -1558,12 +1558,12 @@
       </c>
       <c r="C13" s="29" t="inlineStr">
         <is>
-          <t>The descriptions of the core focus of each unit are clear.</t>
+          <t>The six learning units collectively cover the main competences needed to use AI in on-the-job training.</t>
         </is>
       </c>
       <c r="D13" s="29" t="inlineStr">
         <is>
-          <t>Las descripciones del enfoque central de cada unidad formativa son claras.</t>
+          <t>Las seis unidades de aprendizaje cubren en conjunto las principales competencias necesarias para utilizar la IA en la formación en el puesto de trabajo.</t>
         </is>
       </c>
       <c r="E13" s="28" t="inlineStr">
@@ -1575,7 +1575,7 @@
     <row r="14">
       <c r="A14" s="28" t="inlineStr">
         <is>
-          <t>U3</t>
+          <t>U2</t>
         </is>
       </c>
       <c r="B14" s="29" t="inlineStr">
@@ -1585,12 +1585,12 @@
       </c>
       <c r="C14" s="29" t="inlineStr">
         <is>
-          <t>The main learning outcomes are realistic and appropriate.</t>
+          <t>The descriptions of the core focus of each unit are clear.</t>
         </is>
       </c>
       <c r="D14" s="29" t="inlineStr">
         <is>
-          <t>Los principales resultados de aprendizaje previstos son realistas y adecuados.</t>
+          <t>Las descripciones del enfoque central de cada unidad formativa son claras.</t>
         </is>
       </c>
       <c r="E14" s="28" t="inlineStr">
@@ -1602,7 +1602,7 @@
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
         <is>
-          <t>U4</t>
+          <t>U3</t>
         </is>
       </c>
       <c r="B15" s="29" t="inlineStr">
@@ -1629,7 +1629,7 @@
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
         <is>
-          <t>U5</t>
+          <t>U4</t>
         </is>
       </c>
       <c r="B16" s="29" t="inlineStr">
@@ -1656,22 +1656,22 @@
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
         <is>
-          <t>E1</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="B17" s="29" t="inlineStr">
         <is>
-          <t>Section 5. Ethical, legal and inclusive principles</t>
+          <t>Section 5. Competence framework</t>
         </is>
       </c>
       <c r="C17" s="29" t="inlineStr">
         <is>
-          <t>Ethical and legal aspects are sufficiently integrated into the itinerary.</t>
+          <t>The Knowledge, Skills and Attitudes structure is appropriate for the itinerary.</t>
         </is>
       </c>
       <c r="D17" s="29" t="inlineStr">
         <is>
-          <t>Los aspectos éticos y legales están suficientemente integrados en el itinerario.</t>
+          <t>La estructura de Conocimientos, Habilidades y Actitudes (KSA) es adecuada para el itinerario.</t>
         </is>
       </c>
       <c r="E17" s="28" t="inlineStr">
@@ -1683,22 +1683,22 @@
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
         <is>
-          <t>E2</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B18" s="29" t="inlineStr">
         <is>
-          <t>Section 5. Ethical, legal and inclusive principles</t>
+          <t>Section 5. Competence framework</t>
         </is>
       </c>
       <c r="C18" s="29" t="inlineStr">
         <is>
-          <t>The treatment of ethical and legal issues is appropriate for the target groups.</t>
+          <t>The competence framework is aligned with the learning units.</t>
         </is>
       </c>
       <c r="D18" s="29" t="inlineStr">
         <is>
-          <t>El tratamiento de las cuestiones éticas y legales es adecuado para los grupos destinatarios.</t>
+          <t>El marco de competencias está debidamente alineado con las unidades de aprendizaje.</t>
         </is>
       </c>
       <c r="E18" s="28" t="inlineStr">
@@ -1710,22 +1710,22 @@
     <row r="19">
       <c r="A19" s="28" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="B19" s="29" t="inlineStr">
         <is>
-          <t>Section 5. Ethical, legal and inclusive principles</t>
+          <t>Section 5. Competence framework</t>
         </is>
       </c>
       <c r="C19" s="29" t="inlineStr">
         <is>
-          <t>The ethical dimension is connected meaningfully with tool selection, training design and implementation.</t>
+          <t>The attitudes identified are appropriate for responsible and practical use of AI.</t>
         </is>
       </c>
       <c r="D19" s="29" t="inlineStr">
         <is>
-          <t>La dimensión ética se conecta de forma significativa con la selección de herramientas, el diseño formativo y su ejecución.</t>
+          <t>Las actitudes identificadas son adecuadas para un uso responsable y práctico de la IA.</t>
         </is>
       </c>
       <c r="E19" s="28" t="inlineStr">
@@ -1737,22 +1737,22 @@
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
         <is>
-          <t>E4</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="B20" s="29" t="inlineStr">
         <is>
-          <t>Section 5. Ethical, legal and inclusive principles</t>
+          <t>Section 5. Competence framework</t>
         </is>
       </c>
       <c r="C20" s="29" t="inlineStr">
         <is>
-          <t>The itinerary gives appropriate attention to fairness, accessibility and inclusion.</t>
+          <t>The competence framework can support the subsequent development of learning content and activities.</t>
         </is>
       </c>
       <c r="D20" s="29" t="inlineStr">
         <is>
-          <t>El itinerario presta la debida atención a la equidad, la accesibilidad y la inclusión.</t>
+          <t>El marco de competencias puede sustentar con éxito el posterior desarrollo de contenidos y actividades formativas.</t>
         </is>
       </c>
       <c r="E20" s="28" t="inlineStr">
@@ -1764,22 +1764,22 @@
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="B21" s="29" t="inlineStr">
         <is>
-          <t>Section 6. Competence framework</t>
+          <t>Section 6. Practical use and transferability</t>
         </is>
       </c>
       <c r="C21" s="29" t="inlineStr">
         <is>
-          <t>The Knowledge, Skills and Attitudes structure is appropriate for the itinerary.</t>
+          <t>The itinerary provides useful guidance for developing a complete Training Programme.</t>
         </is>
       </c>
       <c r="D21" s="29" t="inlineStr">
         <is>
-          <t>La estructura de Conocimientos, Habilidades y Actitudes (KSA) es adecuada para el itinerario.</t>
+          <t>El itinerario proporciona directrices útiles para el desarrollo de un Programa Formativo integral.</t>
         </is>
       </c>
       <c r="E21" s="28" t="inlineStr">
@@ -1791,22 +1791,22 @@
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="B22" s="29" t="inlineStr">
         <is>
-          <t>Section 6. Competence framework</t>
+          <t>Section 6. Practical use and transferability</t>
         </is>
       </c>
       <c r="C22" s="29" t="inlineStr">
         <is>
-          <t>The competence framework is aligned with the learning units.</t>
+          <t>The practical guidance for trainers is useful.</t>
         </is>
       </c>
       <c r="D22" s="29" t="inlineStr">
         <is>
-          <t>El marco de competencias está debidamente alineado con las unidades de aprendizaje.</t>
+          <t>Las orientaciones prácticas para formadores son de gran utilidad.</t>
         </is>
       </c>
       <c r="E22" s="28" t="inlineStr">
@@ -1818,22 +1818,22 @@
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="B23" s="29" t="inlineStr">
         <is>
-          <t>Section 6. Competence framework</t>
+          <t>Section 6. Practical use and transferability</t>
         </is>
       </c>
       <c r="C23" s="29" t="inlineStr">
         <is>
-          <t>The attitudes identified are appropriate for responsible and practical use of AI.</t>
+          <t>The adaptation roadmap can help external trainers adapt the itinerary to different learner groups.</t>
         </is>
       </c>
       <c r="D23" s="29" t="inlineStr">
         <is>
-          <t>Las actitudes identificadas son adecuadas para un uso responsable y práctico de la IA.</t>
+          <t>La hoja de ruta de adaptación puede ayudar a formadores externos a adaptar el itinerario a diversos grupos de participantes.</t>
         </is>
       </c>
       <c r="E23" s="28" t="inlineStr">
@@ -1845,22 +1845,22 @@
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>T4</t>
         </is>
       </c>
       <c r="B24" s="29" t="inlineStr">
         <is>
-          <t>Section 6. Competence framework</t>
+          <t>Section 6. Practical use and transferability</t>
         </is>
       </c>
       <c r="C24" s="29" t="inlineStr">
         <is>
-          <t>The competence framework can support the subsequent development of learning content and activities.</t>
+          <t>The itinerary is sufficiently clear to be used by trainers or organisations outside the consortium or beyond the project activities.</t>
         </is>
       </c>
       <c r="D24" s="29" t="inlineStr">
         <is>
-          <t>El marco de competencias puede sustentar con éxito el posterior desarrollo de contenidos y actividades formativas.</t>
+          <t>El itinerario es suficientemente claro como para ser utilizado por formadores u organizaciones ajenas al consorcio o más allá de las actividades del proyecto.</t>
         </is>
       </c>
       <c r="E24" s="28" t="inlineStr">
@@ -1872,22 +1872,22 @@
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T5</t>
         </is>
       </c>
       <c r="B25" s="29" t="inlineStr">
         <is>
-          <t>Section 7. Practical use and transferability</t>
+          <t>Section 6. Practical use and transferability</t>
         </is>
       </c>
       <c r="C25" s="29" t="inlineStr">
         <is>
-          <t>The itinerary provides useful guidance for developing a complete Training Programme.</t>
+          <t>The document has potential to support the development of training actions in different European contexts.</t>
         </is>
       </c>
       <c r="D25" s="29" t="inlineStr">
         <is>
-          <t>El itinerario proporciona directrices útiles para el desarrollo de un Programa Formativo integral.</t>
+          <t>El documento tiene un alto potencial para respaldar el desarrollo de acciones formativas en diversos contextos europeos.</t>
         </is>
       </c>
       <c r="E25" s="28" t="inlineStr">
@@ -1899,22 +1899,22 @@
     <row r="26">
       <c r="A26" s="28" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>E1</t>
         </is>
       </c>
       <c r="B26" s="29" t="inlineStr">
         <is>
-          <t>Section 7. Practical use and transferability</t>
+          <t>Section 7. Ethical, legal and inclusive principles</t>
         </is>
       </c>
       <c r="C26" s="29" t="inlineStr">
         <is>
-          <t>The practical guidance for trainers is useful.</t>
+          <t>Ethical and legal aspects are sufficiently integrated into the itinerary.</t>
         </is>
       </c>
       <c r="D26" s="29" t="inlineStr">
         <is>
-          <t>Las orientaciones prácticas para formadores son de gran utilidad.</t>
+          <t>Los aspectos éticos y legales están suficientemente integrados en el itinerario.</t>
         </is>
       </c>
       <c r="E26" s="28" t="inlineStr">
@@ -1926,22 +1926,22 @@
     <row r="27">
       <c r="A27" s="28" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>E2</t>
         </is>
       </c>
       <c r="B27" s="29" t="inlineStr">
         <is>
-          <t>Section 7. Practical use and transferability</t>
+          <t>Section 7. Ethical, legal and inclusive principles</t>
         </is>
       </c>
       <c r="C27" s="29" t="inlineStr">
         <is>
-          <t>The adaptation roadmap can help external trainers adapt the itinerary to different learner groups.</t>
+          <t>The treatment of ethical and legal issues is appropriate for the target groups.</t>
         </is>
       </c>
       <c r="D27" s="29" t="inlineStr">
         <is>
-          <t>La hoja de ruta de adaptación puede ayudar a formadores externos a adaptar el itinerario a diversos grupos de participantes.</t>
+          <t>El tratamiento de las cuestiones éticas y legales es adecuado para los grupos destinatarios.</t>
         </is>
       </c>
       <c r="E27" s="28" t="inlineStr">
@@ -1953,22 +1953,22 @@
     <row r="28">
       <c r="A28" s="28" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="B28" s="29" t="inlineStr">
         <is>
-          <t>Section 7. Practical use and transferability</t>
+          <t>Section 7. Ethical, legal and inclusive principles</t>
         </is>
       </c>
       <c r="C28" s="29" t="inlineStr">
         <is>
-          <t>The itinerary is sufficiently clear to be used by trainers or organisations outside the consortium or beyond the project activities.</t>
+          <t>The ethical dimension is connected meaningfully with tool selection, training design and implementation.</t>
         </is>
       </c>
       <c r="D28" s="29" t="inlineStr">
         <is>
-          <t>El itinerario es suficientemente claro como para ser utilizado por formadores u organizaciones ajenas al consorcio o más allá de las actividades del proyecto.</t>
+          <t>La dimensión ética se conecta de forma significativa con la selección de herramientas, el diseño formativo y su ejecución.</t>
         </is>
       </c>
       <c r="E28" s="28" t="inlineStr">
@@ -1980,22 +1980,22 @@
     <row r="29">
       <c r="A29" s="28" t="inlineStr">
         <is>
-          <t>T5</t>
+          <t>E4</t>
         </is>
       </c>
       <c r="B29" s="29" t="inlineStr">
         <is>
-          <t>Section 7. Practical use and transferability</t>
+          <t>Section 7. Ethical, legal and inclusive principles</t>
         </is>
       </c>
       <c r="C29" s="29" t="inlineStr">
         <is>
-          <t>The document has potential to support the development of training actions in different European contexts.</t>
+          <t>The itinerary gives appropriate attention to fairness, accessibility and inclusion.</t>
         </is>
       </c>
       <c r="D29" s="29" t="inlineStr">
         <is>
-          <t>El documento tiene un alto potencial para respaldar el desarrollo de acciones formativas en diversos contextos europeos.</t>
+          <t>El itinerario presta la debida atención a la equidad, la accesibilidad y la inclusión.</t>
         </is>
       </c>
       <c r="E29" s="28" t="inlineStr">
@@ -2149,6 +2149,18 @@
       <c r="B40" s="29" t="inlineStr">
         <is>
           <t>Strongly Agree / Totalmente de acuerdo</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="28" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="B41" s="29" t="inlineStr">
+        <is>
+          <t>Not applicable / I cannot assess / No aplicable</t>
         </is>
       </c>
     </row>
@@ -2242,7 +2254,7 @@
       </c>
       <c r="D5" s="40" t="inlineStr">
         <is>
-          <t>Average of items P1 to P4</t>
+          <t>Average of items P1 to P5</t>
         </is>
       </c>
     </row>
@@ -2284,14 +2296,14 @@
       </c>
       <c r="D7" s="40" t="inlineStr">
         <is>
-          <t>Average of items U1 to U5</t>
+          <t>Average of items U1 to U4</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="29" t="inlineStr">
         <is>
-          <t>Section 5: Ethical &amp; Legal Principles Mean</t>
+          <t>Section 5: Competence Framework Mean</t>
         </is>
       </c>
       <c r="B8" s="41">
@@ -2305,14 +2317,14 @@
       </c>
       <c r="D8" s="40" t="inlineStr">
         <is>
-          <t>Average of items E1 to E4</t>
+          <t>Average of items C1 to C4</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="29" t="inlineStr">
         <is>
-          <t>Section 6: Competence Framework Mean</t>
+          <t>Section 6: Practical Use &amp; Transferability Mean</t>
         </is>
       </c>
       <c r="B9" s="41">
@@ -2326,14 +2338,14 @@
       </c>
       <c r="D9" s="40" t="inlineStr">
         <is>
-          <t>Average of items C1 to C4</t>
+          <t>Average of items T1 to T5</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="29" t="inlineStr">
         <is>
-          <t>Section 7: Practical Use &amp; Transferability Mean</t>
+          <t>Section 7: Ethical &amp; Legal Principles Mean</t>
         </is>
       </c>
       <c r="B10" s="41">
@@ -2347,7 +2359,7 @@
       </c>
       <c r="D10" s="40" t="inlineStr">
         <is>
-          <t>Average of items T1 to T5</t>
+          <t>Average of items E1 to E4</t>
         </is>
       </c>
     </row>

</xml_diff>